<commit_message>
git commit -m "fix: adjust LH export close-out style detection"
</commit_message>
<xml_diff>
--- a/APS-Modules/aps-lh/src/main/resources/excelModel/lhjhtemplate.xlsx
+++ b/APS-Modules/aps-lh/src/main/resources/excelModel/lhjhtemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\JY-APS\APS-Modules\aps-lh\src\main\resources\excelModel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\E\CODES\JY_APS\JY_APS_CODE\jy_aps_admin\APS-Modules\aps-lh\src\main\resources\excelModel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D607560-BF16-4A87-A307-A1257CA9D0F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6671925E-A483-4789-B0C7-06909388C31D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="844" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="硫化日计划" sheetId="35" r:id="rId1"/>
@@ -27,10 +27,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -1648,14 +1648,14 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="7">
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="m/d;@"/>
-    <numFmt numFmtId="180" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    <numFmt numFmtId="181" formatCode="[$-409]m/d/yy\ h:mm\ AM/PM;@"/>
-    <numFmt numFmtId="182" formatCode="yyyy/m/d;@"/>
-    <numFmt numFmtId="183" formatCode="[$-10804]0;\(0\)"/>
+    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="m/d;@"/>
+    <numFmt numFmtId="178" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="179" formatCode="[$-409]m/d/yy\ h:mm\ AM/PM;@"/>
+    <numFmt numFmtId="180" formatCode="yyyy/m/d;@"/>
+    <numFmt numFmtId="181" formatCode="[$-10804]0;\(0\)"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <name val="宋体"/>
@@ -1962,15 +1962,15 @@
   </borders>
   <cellStyleXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="178" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="176" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="179" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="178" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -1978,7 +1978,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
-    <xf numFmtId="178" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1987,10 +1987,10 @@
   </cellStyleXfs>
   <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="10" applyFont="1" applyAlignment="1">
@@ -1999,22 +1999,22 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="181" fontId="3" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="1" fillId="0" borderId="2" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="2" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="1" fillId="0" borderId="3" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="3" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2029,7 +2029,7 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="1" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2044,25 +2044,25 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="183" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2083,7 +2083,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="183" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2101,14 +2101,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="183" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2124,12 +2130,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -2594,41 +2594,41 @@
     <tabColor rgb="FF00B050"/>
   </sheetPr>
   <dimension ref="A1:CC6"/>
-  <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="14.25" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="3" width="5.59765625" customWidth="1"/>
+    <col min="1" max="3" width="5.625" customWidth="1"/>
     <col min="4" max="4" width="6.5" customWidth="1"/>
-    <col min="5" max="5" width="9.59765625" customWidth="1"/>
-    <col min="6" max="6" width="32.59765625" customWidth="1"/>
-    <col min="7" max="7" width="9.59765625" customWidth="1"/>
-    <col min="8" max="8" width="32.59765625" customWidth="1"/>
-    <col min="9" max="9" width="17.09765625" customWidth="1"/>
-    <col min="10" max="11" width="5.59765625" customWidth="1"/>
-    <col min="12" max="12" width="6.09765625" customWidth="1"/>
-    <col min="13" max="13" width="5.59765625" customWidth="1"/>
-    <col min="14" max="14" width="3.09765625" customWidth="1"/>
-    <col min="15" max="21" width="5.09765625" customWidth="1"/>
-    <col min="22" max="22" width="3.09765625" customWidth="1"/>
-    <col min="23" max="29" width="5.09765625" customWidth="1"/>
-    <col min="30" max="30" width="3.09765625" customWidth="1"/>
-    <col min="31" max="37" width="5.09765625" customWidth="1"/>
-    <col min="38" max="38" width="3.09765625" customWidth="1"/>
-    <col min="39" max="45" width="5.09765625" customWidth="1"/>
-    <col min="46" max="46" width="3.09765625" customWidth="1"/>
-    <col min="47" max="53" width="5.09765625" customWidth="1"/>
-    <col min="54" max="54" width="3.09765625" customWidth="1"/>
-    <col min="55" max="61" width="5.09765625" customWidth="1"/>
-    <col min="62" max="62" width="3.09765625" customWidth="1"/>
-    <col min="63" max="69" width="5.09765625" customWidth="1"/>
-    <col min="70" max="70" width="3.09765625" customWidth="1"/>
-    <col min="71" max="77" width="5.09765625" customWidth="1"/>
-    <col min="78" max="78" width="9.59765625" customWidth="1"/>
-    <col min="79" max="79" width="7.59765625" customWidth="1"/>
-    <col min="80" max="80" width="9.59765625" customWidth="1"/>
-    <col min="81" max="81" width="25.69921875" customWidth="1"/>
+    <col min="5" max="5" width="9.625" customWidth="1"/>
+    <col min="6" max="6" width="32.625" customWidth="1"/>
+    <col min="7" max="7" width="9.625" customWidth="1"/>
+    <col min="8" max="8" width="32.625" customWidth="1"/>
+    <col min="9" max="9" width="17.125" customWidth="1"/>
+    <col min="10" max="11" width="5.625" customWidth="1"/>
+    <col min="12" max="12" width="6.125" customWidth="1"/>
+    <col min="13" max="13" width="5.625" customWidth="1"/>
+    <col min="14" max="14" width="3.125" customWidth="1"/>
+    <col min="15" max="21" width="5.125" customWidth="1"/>
+    <col min="22" max="22" width="3.125" customWidth="1"/>
+    <col min="23" max="29" width="5.125" customWidth="1"/>
+    <col min="30" max="30" width="3.125" customWidth="1"/>
+    <col min="31" max="37" width="5.125" customWidth="1"/>
+    <col min="38" max="38" width="3.125" customWidth="1"/>
+    <col min="39" max="45" width="5.125" customWidth="1"/>
+    <col min="46" max="46" width="3.125" customWidth="1"/>
+    <col min="47" max="53" width="5.125" customWidth="1"/>
+    <col min="54" max="54" width="3.125" customWidth="1"/>
+    <col min="55" max="61" width="5.125" customWidth="1"/>
+    <col min="62" max="62" width="3.125" customWidth="1"/>
+    <col min="63" max="69" width="5.125" customWidth="1"/>
+    <col min="70" max="70" width="3.125" customWidth="1"/>
+    <col min="71" max="77" width="5.125" customWidth="1"/>
+    <col min="78" max="78" width="9.625" customWidth="1"/>
+    <col min="79" max="79" width="7.625" customWidth="1"/>
+    <col min="80" max="80" width="9.625" customWidth="1"/>
+    <col min="81" max="81" width="25.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:81" hidden="1">
+    <row r="1" spans="1:81" hidden="1" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2873,17 +2873,17 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:81" ht="37.5" customHeight="1">
+    <row r="2" spans="1:81" ht="37.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="17"/>
       <c r="B2" s="17"/>
       <c r="C2" s="17"/>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
       <c r="I2" s="17"/>
       <c r="J2" s="18" t="s">
         <v>82</v>
@@ -2960,7 +2960,7 @@
       <c r="CB2" s="19"/>
       <c r="CC2" s="17"/>
     </row>
-    <row r="3" spans="1:81" ht="16.95" customHeight="1">
+    <row r="3" spans="1:81" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="20">
         <f>SUM(A6:A108139)</f>
         <v>0</v>
@@ -3075,11 +3075,11 @@
       <c r="CB3" s="21"/>
       <c r="CC3" s="21"/>
     </row>
-    <row r="4" spans="1:81" ht="34.200000000000003">
-      <c r="A4" s="43" t="s">
+    <row r="4" spans="1:81" ht="36" x14ac:dyDescent="0.15">
+      <c r="A4" s="45" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="44"/>
+      <c r="B4" s="46"/>
       <c r="C4" s="28" t="s">
         <v>85</v>
       </c>
@@ -3113,86 +3113,86 @@
       <c r="M4" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="N4" s="45" t="s">
+      <c r="N4" s="47" t="s">
         <v>96</v>
       </c>
-      <c r="O4" s="46"/>
-      <c r="P4" s="46"/>
-      <c r="Q4" s="46"/>
-      <c r="R4" s="46"/>
-      <c r="S4" s="46"/>
-      <c r="T4" s="46"/>
-      <c r="U4" s="46"/>
-      <c r="V4" s="45" t="s">
+      <c r="O4" s="48"/>
+      <c r="P4" s="48"/>
+      <c r="Q4" s="48"/>
+      <c r="R4" s="48"/>
+      <c r="S4" s="48"/>
+      <c r="T4" s="48"/>
+      <c r="U4" s="48"/>
+      <c r="V4" s="47" t="s">
         <v>97</v>
       </c>
-      <c r="W4" s="46"/>
-      <c r="X4" s="46"/>
-      <c r="Y4" s="46"/>
-      <c r="Z4" s="46"/>
-      <c r="AA4" s="46"/>
-      <c r="AB4" s="46"/>
-      <c r="AC4" s="46"/>
-      <c r="AD4" s="47" t="s">
+      <c r="W4" s="48"/>
+      <c r="X4" s="48"/>
+      <c r="Y4" s="48"/>
+      <c r="Z4" s="48"/>
+      <c r="AA4" s="48"/>
+      <c r="AB4" s="48"/>
+      <c r="AC4" s="48"/>
+      <c r="AD4" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="AE4" s="47"/>
-      <c r="AF4" s="47"/>
-      <c r="AG4" s="47"/>
-      <c r="AH4" s="47"/>
-      <c r="AI4" s="47"/>
-      <c r="AJ4" s="47"/>
-      <c r="AK4" s="47"/>
-      <c r="AL4" s="47" t="s">
+      <c r="AE4" s="42"/>
+      <c r="AF4" s="42"/>
+      <c r="AG4" s="42"/>
+      <c r="AH4" s="42"/>
+      <c r="AI4" s="42"/>
+      <c r="AJ4" s="42"/>
+      <c r="AK4" s="42"/>
+      <c r="AL4" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="AM4" s="47"/>
-      <c r="AN4" s="47"/>
-      <c r="AO4" s="47"/>
-      <c r="AP4" s="47"/>
-      <c r="AQ4" s="47"/>
-      <c r="AR4" s="47"/>
-      <c r="AS4" s="47"/>
-      <c r="AT4" s="47" t="s">
+      <c r="AM4" s="42"/>
+      <c r="AN4" s="42"/>
+      <c r="AO4" s="42"/>
+      <c r="AP4" s="42"/>
+      <c r="AQ4" s="42"/>
+      <c r="AR4" s="42"/>
+      <c r="AS4" s="42"/>
+      <c r="AT4" s="42" t="s">
         <v>100</v>
       </c>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
-      <c r="AW4" s="47"/>
-      <c r="AX4" s="47"/>
-      <c r="AY4" s="47"/>
-      <c r="AZ4" s="47"/>
-      <c r="BA4" s="47"/>
-      <c r="BB4" s="48" t="s">
+      <c r="AU4" s="42"/>
+      <c r="AV4" s="42"/>
+      <c r="AW4" s="42"/>
+      <c r="AX4" s="42"/>
+      <c r="AY4" s="42"/>
+      <c r="AZ4" s="42"/>
+      <c r="BA4" s="42"/>
+      <c r="BB4" s="43" t="s">
         <v>101</v>
       </c>
-      <c r="BC4" s="48"/>
-      <c r="BD4" s="48"/>
-      <c r="BE4" s="48"/>
-      <c r="BF4" s="48"/>
-      <c r="BG4" s="48"/>
-      <c r="BH4" s="48"/>
-      <c r="BI4" s="48"/>
-      <c r="BJ4" s="48" t="s">
+      <c r="BC4" s="43"/>
+      <c r="BD4" s="43"/>
+      <c r="BE4" s="43"/>
+      <c r="BF4" s="43"/>
+      <c r="BG4" s="43"/>
+      <c r="BH4" s="43"/>
+      <c r="BI4" s="43"/>
+      <c r="BJ4" s="43" t="s">
         <v>102</v>
       </c>
-      <c r="BK4" s="48"/>
-      <c r="BL4" s="48"/>
-      <c r="BM4" s="48"/>
-      <c r="BN4" s="48"/>
-      <c r="BO4" s="48"/>
-      <c r="BP4" s="48"/>
-      <c r="BQ4" s="48"/>
-      <c r="BR4" s="48" t="s">
+      <c r="BK4" s="43"/>
+      <c r="BL4" s="43"/>
+      <c r="BM4" s="43"/>
+      <c r="BN4" s="43"/>
+      <c r="BO4" s="43"/>
+      <c r="BP4" s="43"/>
+      <c r="BQ4" s="43"/>
+      <c r="BR4" s="43" t="s">
         <v>103</v>
       </c>
-      <c r="BS4" s="48"/>
-      <c r="BT4" s="48"/>
-      <c r="BU4" s="48"/>
-      <c r="BV4" s="48"/>
-      <c r="BW4" s="48"/>
-      <c r="BX4" s="48"/>
-      <c r="BY4" s="48"/>
+      <c r="BS4" s="43"/>
+      <c r="BT4" s="43"/>
+      <c r="BU4" s="43"/>
+      <c r="BV4" s="43"/>
+      <c r="BW4" s="43"/>
+      <c r="BX4" s="43"/>
+      <c r="BY4" s="43"/>
       <c r="BZ4" s="28" t="s">
         <v>104</v>
       </c>
@@ -3206,7 +3206,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:81" ht="46.8">
+    <row r="5" spans="1:81" ht="48" x14ac:dyDescent="0.15">
       <c r="A5" s="27" t="s">
         <v>108</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="6" spans="1:81" ht="80.099999999999994" customHeight="1">
+    <row r="6" spans="1:81" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="33" t="s">
         <v>132</v>
       </c>
@@ -3698,16 +3698,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="N4:U4"/>
+    <mergeCell ref="V4:AC4"/>
+    <mergeCell ref="AD4:AK4"/>
     <mergeCell ref="AL4:AS4"/>
     <mergeCell ref="AT4:BA4"/>
     <mergeCell ref="BB4:BI4"/>
     <mergeCell ref="BJ4:BQ4"/>
     <mergeCell ref="BR4:BY4"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="N4:U4"/>
-    <mergeCell ref="V4:AC4"/>
-    <mergeCell ref="AD4:AK4"/>
   </mergeCells>
   <phoneticPr fontId="23" type="noConversion"/>
   <conditionalFormatting sqref="F3:G3">
@@ -3719,8 +3719,8 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3730,25 +3730,25 @@
     <tabColor rgb="FF00B050"/>
   </sheetPr>
   <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultColWidth="8" defaultRowHeight="11.4"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="3" style="3" customWidth="1"/>
-    <col min="2" max="2" width="8.8984375" style="4" customWidth="1"/>
-    <col min="3" max="4" width="5.59765625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="4.69921875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.19921875" style="3" customWidth="1"/>
-    <col min="7" max="7" width="34.09765625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="10.19921875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="34.09765625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="8.69921875" style="5" customWidth="1"/>
-    <col min="11" max="11" width="5.69921875" style="5" customWidth="1"/>
-    <col min="12" max="14" width="5.69921875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="27.3984375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.875" style="4" customWidth="1"/>
+    <col min="3" max="4" width="5.625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="4.75" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.25" style="3" customWidth="1"/>
+    <col min="7" max="7" width="34.125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="10.25" style="3" customWidth="1"/>
+    <col min="9" max="9" width="34.125" style="5" customWidth="1"/>
+    <col min="10" max="10" width="8.75" style="5" customWidth="1"/>
+    <col min="11" max="11" width="5.75" style="5" customWidth="1"/>
+    <col min="12" max="14" width="5.75" style="1" customWidth="1"/>
+    <col min="15" max="15" width="27.375" style="1" customWidth="1"/>
     <col min="16" max="16" width="9" style="1" customWidth="1"/>
     <col min="17" max="16384" width="8" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" hidden="1">
+    <row r="1" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A1" s="3" t="s">
         <v>213</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="33.75" customHeight="1">
+    <row r="2" spans="1:16" ht="33.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="6"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -3818,7 +3818,7 @@
       <c r="O2" s="9"/>
       <c r="P2" s="10"/>
     </row>
-    <row r="3" spans="1:16" s="2" customFormat="1" ht="34.200000000000003" customHeight="1">
+    <row r="3" spans="1:16" s="2" customFormat="1" ht="34.15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="11" t="s">
         <v>229</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:16" s="2" customFormat="1" ht="68.25" customHeight="1">
+    <row r="4" spans="1:16" s="2" customFormat="1" ht="68.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12" t="s">
         <v>242</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="11.4" customHeight="1">
+    <row r="5" spans="1:16" ht="11.45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="13" t="s">
         <v>256</v>
       </c>

</xml_diff>